<commit_message>
fix(lab2): correct experiment workbook formulas
</commit_message>
<xml_diff>
--- a/simulations/lab2/measured/Lab2-數據記錄.xlsx
+++ b/simulations/lab2/measured/Lab2-數據記錄.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第二部分 CE 放大器" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -562,7 +562,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <majorGridlines/>
         <title>
           <tx>
@@ -645,6 +645,9 @@
         <ser>
           <idx val="0"/>
           <order val="0"/>
+          <tx>
+            <v>實測</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -664,6 +667,9 @@
         <ser>
           <idx val="1"/>
           <order val="1"/>
+          <tx>
+            <v>LTspice</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -757,6 +763,9 @@
         <ser>
           <idx val="0"/>
           <order val="0"/>
+          <tx>
+            <v>β</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -815,9 +824,6 @@
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -850,6 +856,9 @@
         <ser>
           <idx val="0"/>
           <order val="0"/>
+          <tx>
+            <v>實測</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -869,6 +878,9 @@
         <ser>
           <idx val="1"/>
           <order val="1"/>
+          <tx>
+            <v>LTspice</v>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -1016,7 +1028,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>9</col>
       <colOff>0</colOff>
       <row>11</row>
       <rowOff>0</rowOff>
@@ -1369,7 +1381,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>每個實驗一張工作表，只要填**黃底**的格子，其他欄位都是公式或預報值，不要覆蓋。</t>
+          <t>每個實驗一張工作表，只要填黃底的格子，其他欄位都是公式或預報值，不要覆蓋。</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1501,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>→ 差異 (%)</t>
+          <t>→ 相對偏差 (%)</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3566,7 @@
       <c r="B51" s="18" t="n"/>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>左表跨 B-E、中表跨 C-E、右表串在 VCC 與 RC 之間</t>
+          <t>左表跨 B-E、中表跨 C-E、右表設 DC 電壓檔並跨 RC 兩端量 V_RC</t>
         </is>
       </c>
     </row>
@@ -3606,6 +3618,11 @@
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="G11:I11"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F11 K11 P11 U11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ON,OFF"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -3637,7 +3654,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>欄位與版面照 App_Lab2.pdf 第 8 頁；數值自動從「實驗一 特性曲線」工作表抓，不要直接在這裡填</t>
+          <t>版面參照 App_Lab2.pdf 第 8 頁；電流統一標示為 mA，數值自動從「實驗一 特性曲線」抓取</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3683,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>I_C (measure)  ( = V_C / R_C )</t>
+          <t>I_C (mA)  ( = V_RC / R_C )</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -3676,7 +3693,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>I_C (measure)  ( = V_C / R_C )</t>
+          <t>I_C (mA)  ( = V_RC / R_C )</t>
         </is>
       </c>
       <c r="H6" s="6" t="n">
@@ -3810,7 +3827,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>I_C (measure)  ( = V_C / R_C )</t>
+          <t>I_C (mA)  ( = V_RC / R_C )</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -3820,7 +3837,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>I_C (measure)  ( = V_C / R_C )</t>
+          <t>I_C (mA)  ( = V_RC / R_C )</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3934,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>I_C 的單位是 mA（講義表頭寫 A，抄進報告時記得換算或標註單位）。</t>
+          <t>I_C 已統一使用 mA；若指定報告格式要求 A，請將數值除以 1000 並同步標註單位。</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4079,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>差異 (%)</t>
+          <t>相對偏差 (%)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -4190,9 +4207,10 @@
           <t>mA</t>
         </is>
       </c>
-      <c r="D11" s="19">
-        <f>IF(B7="","",B7/$C$4*1000)</f>
-        <v/>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>V_R1 ÷ R1 × 1000</t>
+        </is>
       </c>
       <c r="E11" s="9" t="n">
         <v>1.425</v>
@@ -4222,9 +4240,10 @@
           <t>mA</t>
         </is>
       </c>
-      <c r="D12" s="19">
-        <f>IF(B8="","",B8/$E$4*1000)</f>
-        <v/>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>V_R2 ÷ R2 × 1000</t>
+        </is>
       </c>
       <c r="E12" s="9" t="n">
         <v>0.159</v>
@@ -4254,9 +4273,10 @@
           <t>mA</t>
         </is>
       </c>
-      <c r="D13" s="19">
-        <f>IF(OR(B7="",B8=""),"",B11-B12)</f>
-        <v/>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>I_R1 − I_R2</t>
+        </is>
       </c>
       <c r="E13" s="9" t="n">
         <v>1.266</v>
@@ -4286,9 +4306,10 @@
           <t>mA</t>
         </is>
       </c>
-      <c r="D14" s="19">
-        <f>IF(B9="","",B9/$G$4*1000)</f>
-        <v/>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>V_RC ÷ R_C × 1000</t>
+        </is>
       </c>
       <c r="E14" s="9" t="n">
         <v>14.946</v>
@@ -4318,9 +4339,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D15" s="19">
-        <f>IF(OR(B13="",B13=0,B14=""),"",B14/B13)</f>
-        <v/>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>I_C ÷ I_B</t>
+        </is>
       </c>
       <c r="E15" s="9" t="n">
         <v>11.81</v>
@@ -4471,7 +4493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4481,6 +4503,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4497,6 +4520,37 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>直流計算設定</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>V_CC (V)</t>
+        </is>
+      </c>
+      <c r="C3" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>R_C1 100 Ω 實測 (Ω)</t>
+        </is>
+      </c>
+      <c r="E3" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>R_C1 1 kΩ 實測 (Ω)</t>
+        </is>
+      </c>
+      <c r="G3" s="23" t="n">
+        <v>1000</v>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4512,7 +4566,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>實測 (V)</t>
+          <t>實測 R_C1 = 100 Ω</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -4522,20 +4576,29 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
+          <t>相對偏差 (%)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>實測 R_C1 = 1 kΩ</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>LTspice R_C1 = 1 kΩ</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>差異 (%)</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>相對偏差 (%)</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
@@ -4547,14 +4610,19 @@
       <c r="C6" s="9" t="n">
         <v>5.876</v>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="10">
+        <f>IF(OR(B6="",C6=0),"",(B6-C6)/C6)</f>
+        <v/>
+      </c>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="9" t="n">
         <v>5.87</v>
       </c>
-      <c r="E6" s="10">
-        <f>IF(OR(B6="",C6=0),"",(B6-C6)/C6)</f>
-        <v/>
-      </c>
-      <c r="F6" s="19" t="inlineStr">
+      <c r="G6" s="10">
+        <f>IF(OR(E6="",F6=0),"",(E6-F6)/F6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
         <is>
           <t>分壓器給的 6 V 附近</t>
         </is>
@@ -4570,14 +4638,19 @@
       <c r="C7" s="9" t="n">
         <v>5.178</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="10">
+        <f>IF(OR(B7="",C7=0),"",(B7-C7)/C7)</f>
+        <v/>
+      </c>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="9" t="n">
         <v>5.171</v>
       </c>
-      <c r="E7" s="10">
-        <f>IF(OR(B7="",C7=0),"",(B7-C7)/C7)</f>
-        <v/>
-      </c>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="G7" s="10">
+        <f>IF(OR(E7="",F7=0),"",(E7-F7)/F7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>約 V_B − 0.7</t>
         </is>
@@ -4593,14 +4666,19 @@
       <c r="C8" s="9" t="n">
         <v>11.485</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="10">
+        <f>IF(OR(B8="",C8=0),"",(B8-C8)/C8)</f>
+        <v/>
+      </c>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="9" t="n">
         <v>6.854</v>
       </c>
-      <c r="E8" s="10">
-        <f>IF(OR(B8="",C8=0),"",(B8-C8)/C8)</f>
-        <v/>
-      </c>
-      <c r="F8" s="19" t="inlineStr">
+      <c r="G8" s="10">
+        <f>IF(OR(E8="",F8=0),"",(E8-F8)/F8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
         <is>
           <t>R_C1 越大這裡越低</t>
         </is>
@@ -4612,20 +4690,31 @@
           <t>V_CE = V_C − V_E</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
+      <c r="B9" s="8">
+        <f>IF(OR(B7="",B8=""),"",B8-B7)</f>
+        <v/>
+      </c>
       <c r="C9" s="9" t="n">
         <v>6.306</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="10">
+        <f>IF(OR(B9="",C9=0),"",(B9-C9)/C9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="8">
+        <f>IF(OR(E7="",E8=""),"",E8-E7)</f>
+        <v/>
+      </c>
+      <c r="F9" s="9" t="n">
         <v>1.683</v>
       </c>
-      <c r="E9" s="10">
-        <f>IF(OR(B9="",C9=0),"",(B9-C9)/C9)</f>
-        <v/>
-      </c>
-      <c r="F9" s="19" t="inlineStr">
-        <is>
-          <t>小於 1 V 就代表快飽和，訊號會削波</t>
+      <c r="G9" s="10">
+        <f>IF(OR(E9="",F9=0),"",(E9-F9)/F9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>由 V_C − V_E 自動計算；小於 1 V 就代表快飽和，訊號會削波</t>
         </is>
       </c>
     </row>
@@ -4636,19 +4725,30 @@
         </is>
       </c>
       <c r="B10" s="8">
-        <f>IF(B8="","",(12-B8)/100*1000)</f>
+        <f>IF(OR(B8="",$C$3="",$E$3="",$E$3=0),"",($C$3-B8)/$E$3*1000)</f>
         <v/>
       </c>
       <c r="C10" s="9" t="n">
         <v>5.153</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="10">
+        <f>IF(OR(B10="",C10=0),"",(B10-C10)/C10)</f>
+        <v/>
+      </c>
+      <c r="E10" s="8">
+        <f>IF(OR(E8="",$C$3="",$G$3="",$G$3=0),"",($C$3-E8)/$G$3*1000)</f>
+        <v/>
+      </c>
+      <c r="F10" s="9" t="n">
         <v>5.146</v>
       </c>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="19" t="inlineStr">
-        <is>
-          <t>單位 mA；式子裡的 100 要跟著實際用的 R_C1 改</t>
+      <c r="G10" s="10">
+        <f>IF(OR(E10="",F10=0),"",(E10-F10)/F10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>單位 mA；使用上方輸入的 V_CC 與兩顆 R_C1 實測阻值計算</t>
         </is>
       </c>
     </row>
@@ -4677,7 +4777,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>|A_v| = V_out / V_s</t>
+          <t>實測 |A_v| (= V_out/V_s)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -4687,7 +4787,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>差異 (%)</t>
+          <t>相對偏差 (%)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -5047,8 +5147,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
fix(lab2): keep measurement inputs blank
</commit_message>
<xml_diff>
--- a/simulations/lab2/measured/Lab2-數據記錄.xlsx
+++ b/simulations/lab2/measured/Lab2-數據記錄.xlsx
@@ -1726,8 +1726,8 @@
       </c>
       <c r="C11" s="14" t="n"/>
       <c r="D11" s="14" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="15" t="n"/>
+      <c r="E11" s="7" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
       <c r="G11" s="13" t="inlineStr">
         <is>
           <t>V_BB = 2.0 V　V_BE =</t>
@@ -1735,8 +1735,8 @@
       </c>
       <c r="H11" s="14" t="n"/>
       <c r="I11" s="14" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="15" t="n"/>
+      <c r="J11" s="7" t="inlineStr"/>
+      <c r="K11" s="15" t="inlineStr"/>
       <c r="L11" s="13" t="inlineStr">
         <is>
           <t>V_BB = 2.2 V　V_BE =</t>
@@ -1744,8 +1744,8 @@
       </c>
       <c r="M11" s="14" t="n"/>
       <c r="N11" s="14" t="n"/>
-      <c r="O11" s="7" t="n"/>
-      <c r="P11" s="15" t="n"/>
+      <c r="O11" s="7" t="inlineStr"/>
+      <c r="P11" s="15" t="inlineStr"/>
       <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>V_BB = 2.4 V　V_BE =</t>
@@ -1753,8 +1753,8 @@
       </c>
       <c r="R11" s="14" t="n"/>
       <c r="S11" s="14" t="n"/>
-      <c r="T11" s="7" t="n"/>
-      <c r="U11" s="15" t="n"/>
+      <c r="T11" s="7" t="inlineStr"/>
+      <c r="U11" s="15" t="inlineStr"/>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1867,8 +1867,8 @@
       <c r="A13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
+      <c r="B13" s="7" t="inlineStr"/>
+      <c r="C13" s="7" t="inlineStr"/>
       <c r="D13" s="8">
         <f>IF(C13&lt;&gt;"",C13/$B$4*1000,IF(B13&lt;&gt;"",($A13-B13)/$B$4*1000,""))</f>
         <v/>
@@ -1879,8 +1879,8 @@
       <c r="F13" s="9" t="n">
         <v>-0.0003</v>
       </c>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
+      <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr"/>
       <c r="I13" s="8">
         <f>IF(H13&lt;&gt;"",H13/$B$4*1000,IF(G13&lt;&gt;"",($A13-G13)/$B$4*1000,""))</f>
         <v/>
@@ -1891,8 +1891,8 @@
       <c r="K13" s="9" t="n">
         <v>-0.0054</v>
       </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
+      <c r="L13" s="7" t="inlineStr"/>
+      <c r="M13" s="7" t="inlineStr"/>
       <c r="N13" s="8">
         <f>IF(M13&lt;&gt;"",M13/$B$4*1000,IF(L13&lt;&gt;"",($A13-L13)/$B$4*1000,""))</f>
         <v/>
@@ -1903,8 +1903,8 @@
       <c r="P13" s="9" t="n">
         <v>-0.0062</v>
       </c>
-      <c r="Q13" s="7" t="n"/>
-      <c r="R13" s="7" t="n"/>
+      <c r="Q13" s="7" t="inlineStr"/>
+      <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="8">
         <f>IF(R13&lt;&gt;"",R13/$B$4*1000,IF(Q13&lt;&gt;"",($A13-Q13)/$B$4*1000,""))</f>
         <v/>
@@ -1920,8 +1920,8 @@
       <c r="A14" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
+      <c r="B14" s="7" t="inlineStr"/>
+      <c r="C14" s="7" t="inlineStr"/>
       <c r="D14" s="8">
         <f>IF(C14&lt;&gt;"",C14/$B$4*1000,IF(B14&lt;&gt;"",($A14-B14)/$B$4*1000,""))</f>
         <v/>
@@ -1932,8 +1932,8 @@
       <c r="F14" s="9" t="n">
         <v>0.0011</v>
       </c>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="7" t="n"/>
+      <c r="G14" s="7" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr"/>
       <c r="I14" s="8">
         <f>IF(H14&lt;&gt;"",H14/$B$4*1000,IF(G14&lt;&gt;"",($A14-G14)/$B$4*1000,""))</f>
         <v/>
@@ -1944,8 +1944,8 @@
       <c r="K14" s="9" t="n">
         <v>0.3741</v>
       </c>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7" t="n"/>
+      <c r="L14" s="7" t="inlineStr"/>
+      <c r="M14" s="7" t="inlineStr"/>
       <c r="N14" s="8">
         <f>IF(M14&lt;&gt;"",M14/$B$4*1000,IF(L14&lt;&gt;"",($A14-L14)/$B$4*1000,""))</f>
         <v/>
@@ -1956,8 +1956,8 @@
       <c r="P14" s="9" t="n">
         <v>0.4411</v>
       </c>
-      <c r="Q14" s="7" t="n"/>
-      <c r="R14" s="7" t="n"/>
+      <c r="Q14" s="7" t="inlineStr"/>
+      <c r="R14" s="7" t="inlineStr"/>
       <c r="S14" s="8">
         <f>IF(R14&lt;&gt;"",R14/$B$4*1000,IF(Q14&lt;&gt;"",($A14-Q14)/$B$4*1000,""))</f>
         <v/>
@@ -1973,8 +1973,8 @@
       <c r="A15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
+      <c r="B15" s="7" t="inlineStr"/>
+      <c r="C15" s="7" t="inlineStr"/>
       <c r="D15" s="8">
         <f>IF(C15&lt;&gt;"",C15/$B$4*1000,IF(B15&lt;&gt;"",($A15-B15)/$B$4*1000,""))</f>
         <v/>
@@ -1985,8 +1985,8 @@
       <c r="F15" s="9" t="n">
         <v>0.0011</v>
       </c>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="7" t="n"/>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
       <c r="I15" s="8">
         <f>IF(H15&lt;&gt;"",H15/$B$4*1000,IF(G15&lt;&gt;"",($A15-G15)/$B$4*1000,""))</f>
         <v/>
@@ -1997,8 +1997,8 @@
       <c r="K15" s="9" t="n">
         <v>0.4186</v>
       </c>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
+      <c r="L15" s="7" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr"/>
       <c r="N15" s="8">
         <f>IF(M15&lt;&gt;"",M15/$B$4*1000,IF(L15&lt;&gt;"",($A15-L15)/$B$4*1000,""))</f>
         <v/>
@@ -2009,8 +2009,8 @@
       <c r="P15" s="9" t="n">
         <v>0.9111</v>
       </c>
-      <c r="Q15" s="7" t="n"/>
-      <c r="R15" s="7" t="n"/>
+      <c r="Q15" s="7" t="inlineStr"/>
+      <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="8">
         <f>IF(R15&lt;&gt;"",R15/$B$4*1000,IF(Q15&lt;&gt;"",($A15-Q15)/$B$4*1000,""))</f>
         <v/>
@@ -2026,8 +2026,8 @@
       <c r="A16" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
+      <c r="B16" s="7" t="inlineStr"/>
+      <c r="C16" s="7" t="inlineStr"/>
       <c r="D16" s="8">
         <f>IF(C16&lt;&gt;"",C16/$B$4*1000,IF(B16&lt;&gt;"",($A16-B16)/$B$4*1000,""))</f>
         <v/>
@@ -2038,8 +2038,8 @@
       <c r="F16" s="9" t="n">
         <v>0.0011</v>
       </c>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="7" t="n"/>
+      <c r="G16" s="7" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr"/>
       <c r="I16" s="8">
         <f>IF(H16&lt;&gt;"",H16/$B$4*1000,IF(G16&lt;&gt;"",($A16-G16)/$B$4*1000,""))</f>
         <v/>
@@ -2050,8 +2050,8 @@
       <c r="K16" s="9" t="n">
         <v>0.4207</v>
       </c>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
+      <c r="L16" s="7" t="inlineStr"/>
+      <c r="M16" s="7" t="inlineStr"/>
       <c r="N16" s="8">
         <f>IF(M16&lt;&gt;"",M16/$B$4*1000,IF(L16&lt;&gt;"",($A16-L16)/$B$4*1000,""))</f>
         <v/>
@@ -2062,8 +2062,8 @@
       <c r="P16" s="9" t="n">
         <v>1.3821</v>
       </c>
-      <c r="Q16" s="7" t="n"/>
-      <c r="R16" s="7" t="n"/>
+      <c r="Q16" s="7" t="inlineStr"/>
+      <c r="R16" s="7" t="inlineStr"/>
       <c r="S16" s="8">
         <f>IF(R16&lt;&gt;"",R16/$B$4*1000,IF(Q16&lt;&gt;"",($A16-Q16)/$B$4*1000,""))</f>
         <v/>
@@ -2079,8 +2079,8 @@
       <c r="A17" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
+      <c r="B17" s="7" t="inlineStr"/>
+      <c r="C17" s="7" t="inlineStr"/>
       <c r="D17" s="8">
         <f>IF(C17&lt;&gt;"",C17/$B$4*1000,IF(B17&lt;&gt;"",($A17-B17)/$B$4*1000,""))</f>
         <v/>
@@ -2091,8 +2091,8 @@
       <c r="F17" s="9" t="n">
         <v>0.0011</v>
       </c>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
+      <c r="G17" s="7" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr"/>
       <c r="I17" s="8">
         <f>IF(H17&lt;&gt;"",H17/$B$4*1000,IF(G17&lt;&gt;"",($A17-G17)/$B$4*1000,""))</f>
         <v/>
@@ -2103,8 +2103,8 @@
       <c r="K17" s="9" t="n">
         <v>0.4228</v>
       </c>
-      <c r="L17" s="7" t="n"/>
-      <c r="M17" s="7" t="n"/>
+      <c r="L17" s="7" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr"/>
       <c r="N17" s="8">
         <f>IF(M17&lt;&gt;"",M17/$B$4*1000,IF(L17&lt;&gt;"",($A17-L17)/$B$4*1000,""))</f>
         <v/>
@@ -2115,8 +2115,8 @@
       <c r="P17" s="9" t="n">
         <v>1.8252</v>
       </c>
-      <c r="Q17" s="7" t="n"/>
-      <c r="R17" s="7" t="n"/>
+      <c r="Q17" s="7" t="inlineStr"/>
+      <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="8">
         <f>IF(R17&lt;&gt;"",R17/$B$4*1000,IF(Q17&lt;&gt;"",($A17-Q17)/$B$4*1000,""))</f>
         <v/>
@@ -2132,8 +2132,8 @@
       <c r="A18" s="6" t="n">
         <v>2.5</v>
       </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
+      <c r="B18" s="7" t="inlineStr"/>
+      <c r="C18" s="7" t="inlineStr"/>
       <c r="D18" s="8">
         <f>IF(C18&lt;&gt;"",C18/$B$4*1000,IF(B18&lt;&gt;"",($A18-B18)/$B$4*1000,""))</f>
         <v/>
@@ -2144,8 +2144,8 @@
       <c r="F18" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
+      <c r="G18" s="7" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr"/>
       <c r="I18" s="8">
         <f>IF(H18&lt;&gt;"",H18/$B$4*1000,IF(G18&lt;&gt;"",($A18-G18)/$B$4*1000,""))</f>
         <v/>
@@ -2156,8 +2156,8 @@
       <c r="K18" s="9" t="n">
         <v>0.4249</v>
       </c>
-      <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="n"/>
+      <c r="L18" s="7" t="inlineStr"/>
+      <c r="M18" s="7" t="inlineStr"/>
       <c r="N18" s="8">
         <f>IF(M18&lt;&gt;"",M18/$B$4*1000,IF(L18&lt;&gt;"",($A18-L18)/$B$4*1000,""))</f>
         <v/>
@@ -2168,8 +2168,8 @@
       <c r="P18" s="9" t="n">
         <v>1.9141</v>
       </c>
-      <c r="Q18" s="7" t="n"/>
-      <c r="R18" s="7" t="n"/>
+      <c r="Q18" s="7" t="inlineStr"/>
+      <c r="R18" s="7" t="inlineStr"/>
       <c r="S18" s="8">
         <f>IF(R18&lt;&gt;"",R18/$B$4*1000,IF(Q18&lt;&gt;"",($A18-Q18)/$B$4*1000,""))</f>
         <v/>
@@ -2185,8 +2185,8 @@
       <c r="A19" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
+      <c r="B19" s="7" t="inlineStr"/>
+      <c r="C19" s="7" t="inlineStr"/>
       <c r="D19" s="8">
         <f>IF(C19&lt;&gt;"",C19/$B$4*1000,IF(B19&lt;&gt;"",($A19-B19)/$B$4*1000,""))</f>
         <v/>
@@ -2197,8 +2197,8 @@
       <c r="F19" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
+      <c r="G19" s="7" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr"/>
       <c r="I19" s="8">
         <f>IF(H19&lt;&gt;"",H19/$B$4*1000,IF(G19&lt;&gt;"",($A19-G19)/$B$4*1000,""))</f>
         <v/>
@@ -2209,8 +2209,8 @@
       <c r="K19" s="9" t="n">
         <v>0.4269</v>
       </c>
-      <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
+      <c r="L19" s="7" t="inlineStr"/>
+      <c r="M19" s="7" t="inlineStr"/>
       <c r="N19" s="8">
         <f>IF(M19&lt;&gt;"",M19/$B$4*1000,IF(L19&lt;&gt;"",($A19-L19)/$B$4*1000,""))</f>
         <v/>
@@ -2221,8 +2221,8 @@
       <c r="P19" s="9" t="n">
         <v>1.9234</v>
       </c>
-      <c r="Q19" s="7" t="n"/>
-      <c r="R19" s="7" t="n"/>
+      <c r="Q19" s="7" t="inlineStr"/>
+      <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="8">
         <f>IF(R19&lt;&gt;"",R19/$B$4*1000,IF(Q19&lt;&gt;"",($A19-Q19)/$B$4*1000,""))</f>
         <v/>
@@ -2238,8 +2238,8 @@
       <c r="A20" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
+      <c r="B20" s="7" t="inlineStr"/>
+      <c r="C20" s="7" t="inlineStr"/>
       <c r="D20" s="8">
         <f>IF(C20&lt;&gt;"",C20/$B$4*1000,IF(B20&lt;&gt;"",($A20-B20)/$B$4*1000,""))</f>
         <v/>
@@ -2250,8 +2250,8 @@
       <c r="F20" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
+      <c r="G20" s="7" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr"/>
       <c r="I20" s="8">
         <f>IF(H20&lt;&gt;"",H20/$B$4*1000,IF(G20&lt;&gt;"",($A20-G20)/$B$4*1000,""))</f>
         <v/>
@@ -2262,8 +2262,8 @@
       <c r="K20" s="9" t="n">
         <v>0.429</v>
       </c>
-      <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
+      <c r="L20" s="7" t="inlineStr"/>
+      <c r="M20" s="7" t="inlineStr"/>
       <c r="N20" s="8">
         <f>IF(M20&lt;&gt;"",M20/$B$4*1000,IF(L20&lt;&gt;"",($A20-L20)/$B$4*1000,""))</f>
         <v/>
@@ -2274,8 +2274,8 @@
       <c r="P20" s="9" t="n">
         <v>1.9328</v>
       </c>
-      <c r="Q20" s="7" t="n"/>
-      <c r="R20" s="7" t="n"/>
+      <c r="Q20" s="7" t="inlineStr"/>
+      <c r="R20" s="7" t="inlineStr"/>
       <c r="S20" s="8">
         <f>IF(R20&lt;&gt;"",R20/$B$4*1000,IF(Q20&lt;&gt;"",($A20-Q20)/$B$4*1000,""))</f>
         <v/>
@@ -2291,8 +2291,8 @@
       <c r="A21" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
+      <c r="B21" s="7" t="inlineStr"/>
+      <c r="C21" s="7" t="inlineStr"/>
       <c r="D21" s="8">
         <f>IF(C21&lt;&gt;"",C21/$B$4*1000,IF(B21&lt;&gt;"",($A21-B21)/$B$4*1000,""))</f>
         <v/>
@@ -2303,8 +2303,8 @@
       <c r="F21" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
+      <c r="G21" s="7" t="inlineStr"/>
+      <c r="H21" s="7" t="inlineStr"/>
       <c r="I21" s="8">
         <f>IF(H21&lt;&gt;"",H21/$B$4*1000,IF(G21&lt;&gt;"",($A21-G21)/$B$4*1000,""))</f>
         <v/>
@@ -2315,8 +2315,8 @@
       <c r="K21" s="9" t="n">
         <v>0.4311</v>
       </c>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
+      <c r="L21" s="7" t="inlineStr"/>
+      <c r="M21" s="7" t="inlineStr"/>
       <c r="N21" s="8">
         <f>IF(M21&lt;&gt;"",M21/$B$4*1000,IF(L21&lt;&gt;"",($A21-L21)/$B$4*1000,""))</f>
         <v/>
@@ -2327,8 +2327,8 @@
       <c r="P21" s="9" t="n">
         <v>1.9421</v>
       </c>
-      <c r="Q21" s="7" t="n"/>
-      <c r="R21" s="7" t="n"/>
+      <c r="Q21" s="7" t="inlineStr"/>
+      <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="8">
         <f>IF(R21&lt;&gt;"",R21/$B$4*1000,IF(Q21&lt;&gt;"",($A21-Q21)/$B$4*1000,""))</f>
         <v/>
@@ -2344,8 +2344,8 @@
       <c r="A22" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
+      <c r="B22" s="7" t="inlineStr"/>
+      <c r="C22" s="7" t="inlineStr"/>
       <c r="D22" s="8">
         <f>IF(C22&lt;&gt;"",C22/$B$4*1000,IF(B22&lt;&gt;"",($A22-B22)/$B$4*1000,""))</f>
         <v/>
@@ -2356,8 +2356,8 @@
       <c r="F22" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
+      <c r="G22" s="7" t="inlineStr"/>
+      <c r="H22" s="7" t="inlineStr"/>
       <c r="I22" s="8">
         <f>IF(H22&lt;&gt;"",H22/$B$4*1000,IF(G22&lt;&gt;"",($A22-G22)/$B$4*1000,""))</f>
         <v/>
@@ -2368,8 +2368,8 @@
       <c r="K22" s="9" t="n">
         <v>0.4332</v>
       </c>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
+      <c r="L22" s="7" t="inlineStr"/>
+      <c r="M22" s="7" t="inlineStr"/>
       <c r="N22" s="8">
         <f>IF(M22&lt;&gt;"",M22/$B$4*1000,IF(L22&lt;&gt;"",($A22-L22)/$B$4*1000,""))</f>
         <v/>
@@ -2380,8 +2380,8 @@
       <c r="P22" s="9" t="n">
         <v>1.9514</v>
       </c>
-      <c r="Q22" s="7" t="n"/>
-      <c r="R22" s="7" t="n"/>
+      <c r="Q22" s="7" t="inlineStr"/>
+      <c r="R22" s="7" t="inlineStr"/>
       <c r="S22" s="8">
         <f>IF(R22&lt;&gt;"",R22/$B$4*1000,IF(Q22&lt;&gt;"",($A22-Q22)/$B$4*1000,""))</f>
         <v/>
@@ -2397,8 +2397,8 @@
       <c r="A23" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
+      <c r="B23" s="7" t="inlineStr"/>
+      <c r="C23" s="7" t="inlineStr"/>
       <c r="D23" s="8">
         <f>IF(C23&lt;&gt;"",C23/$B$4*1000,IF(B23&lt;&gt;"",($A23-B23)/$B$4*1000,""))</f>
         <v/>
@@ -2409,8 +2409,8 @@
       <c r="F23" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="7" t="n"/>
+      <c r="G23" s="7" t="inlineStr"/>
+      <c r="H23" s="7" t="inlineStr"/>
       <c r="I23" s="8">
         <f>IF(H23&lt;&gt;"",H23/$B$4*1000,IF(G23&lt;&gt;"",($A23-G23)/$B$4*1000,""))</f>
         <v/>
@@ -2421,8 +2421,8 @@
       <c r="K23" s="9" t="n">
         <v>0.4353</v>
       </c>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="n"/>
+      <c r="L23" s="7" t="inlineStr"/>
+      <c r="M23" s="7" t="inlineStr"/>
       <c r="N23" s="8">
         <f>IF(M23&lt;&gt;"",M23/$B$4*1000,IF(L23&lt;&gt;"",($A23-L23)/$B$4*1000,""))</f>
         <v/>
@@ -2433,8 +2433,8 @@
       <c r="P23" s="9" t="n">
         <v>1.9608</v>
       </c>
-      <c r="Q23" s="7" t="n"/>
-      <c r="R23" s="7" t="n"/>
+      <c r="Q23" s="7" t="inlineStr"/>
+      <c r="R23" s="7" t="inlineStr"/>
       <c r="S23" s="8">
         <f>IF(R23&lt;&gt;"",R23/$B$4*1000,IF(Q23&lt;&gt;"",($A23-Q23)/$B$4*1000,""))</f>
         <v/>
@@ -2450,8 +2450,8 @@
       <c r="A24" s="6" t="n">
         <v>5.5</v>
       </c>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="n"/>
+      <c r="B24" s="7" t="inlineStr"/>
+      <c r="C24" s="7" t="inlineStr"/>
       <c r="D24" s="8">
         <f>IF(C24&lt;&gt;"",C24/$B$4*1000,IF(B24&lt;&gt;"",($A24-B24)/$B$4*1000,""))</f>
         <v/>
@@ -2462,8 +2462,8 @@
       <c r="F24" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="7" t="n"/>
+      <c r="G24" s="7" t="inlineStr"/>
+      <c r="H24" s="7" t="inlineStr"/>
       <c r="I24" s="8">
         <f>IF(H24&lt;&gt;"",H24/$B$4*1000,IF(G24&lt;&gt;"",($A24-G24)/$B$4*1000,""))</f>
         <v/>
@@ -2474,8 +2474,8 @@
       <c r="K24" s="9" t="n">
         <v>0.4373</v>
       </c>
-      <c r="L24" s="7" t="n"/>
-      <c r="M24" s="7" t="n"/>
+      <c r="L24" s="7" t="inlineStr"/>
+      <c r="M24" s="7" t="inlineStr"/>
       <c r="N24" s="8">
         <f>IF(M24&lt;&gt;"",M24/$B$4*1000,IF(L24&lt;&gt;"",($A24-L24)/$B$4*1000,""))</f>
         <v/>
@@ -2486,8 +2486,8 @@
       <c r="P24" s="9" t="n">
         <v>1.9701</v>
       </c>
-      <c r="Q24" s="7" t="n"/>
-      <c r="R24" s="7" t="n"/>
+      <c r="Q24" s="7" t="inlineStr"/>
+      <c r="R24" s="7" t="inlineStr"/>
       <c r="S24" s="8">
         <f>IF(R24&lt;&gt;"",R24/$B$4*1000,IF(Q24&lt;&gt;"",($A24-Q24)/$B$4*1000,""))</f>
         <v/>
@@ -2503,8 +2503,8 @@
       <c r="A25" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="n"/>
+      <c r="B25" s="7" t="inlineStr"/>
+      <c r="C25" s="7" t="inlineStr"/>
       <c r="D25" s="8">
         <f>IF(C25&lt;&gt;"",C25/$B$4*1000,IF(B25&lt;&gt;"",($A25-B25)/$B$4*1000,""))</f>
         <v/>
@@ -2515,8 +2515,8 @@
       <c r="F25" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
+      <c r="G25" s="7" t="inlineStr"/>
+      <c r="H25" s="7" t="inlineStr"/>
       <c r="I25" s="8">
         <f>IF(H25&lt;&gt;"",H25/$B$4*1000,IF(G25&lt;&gt;"",($A25-G25)/$B$4*1000,""))</f>
         <v/>
@@ -2527,8 +2527,8 @@
       <c r="K25" s="9" t="n">
         <v>0.4394</v>
       </c>
-      <c r="L25" s="7" t="n"/>
-      <c r="M25" s="7" t="n"/>
+      <c r="L25" s="7" t="inlineStr"/>
+      <c r="M25" s="7" t="inlineStr"/>
       <c r="N25" s="8">
         <f>IF(M25&lt;&gt;"",M25/$B$4*1000,IF(L25&lt;&gt;"",($A25-L25)/$B$4*1000,""))</f>
         <v/>
@@ -2539,8 +2539,8 @@
       <c r="P25" s="9" t="n">
         <v>1.9794</v>
       </c>
-      <c r="Q25" s="7" t="n"/>
-      <c r="R25" s="7" t="n"/>
+      <c r="Q25" s="7" t="inlineStr"/>
+      <c r="R25" s="7" t="inlineStr"/>
       <c r="S25" s="8">
         <f>IF(R25&lt;&gt;"",R25/$B$4*1000,IF(Q25&lt;&gt;"",($A25-Q25)/$B$4*1000,""))</f>
         <v/>
@@ -2556,8 +2556,8 @@
       <c r="A26" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
+      <c r="B26" s="7" t="inlineStr"/>
+      <c r="C26" s="7" t="inlineStr"/>
       <c r="D26" s="8">
         <f>IF(C26&lt;&gt;"",C26/$B$4*1000,IF(B26&lt;&gt;"",($A26-B26)/$B$4*1000,""))</f>
         <v/>
@@ -2568,8 +2568,8 @@
       <c r="F26" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="7" t="n"/>
+      <c r="G26" s="7" t="inlineStr"/>
+      <c r="H26" s="7" t="inlineStr"/>
       <c r="I26" s="8">
         <f>IF(H26&lt;&gt;"",H26/$B$4*1000,IF(G26&lt;&gt;"",($A26-G26)/$B$4*1000,""))</f>
         <v/>
@@ -2580,8 +2580,8 @@
       <c r="K26" s="9" t="n">
         <v>0.4415</v>
       </c>
-      <c r="L26" s="7" t="n"/>
-      <c r="M26" s="7" t="n"/>
+      <c r="L26" s="7" t="inlineStr"/>
+      <c r="M26" s="7" t="inlineStr"/>
       <c r="N26" s="8">
         <f>IF(M26&lt;&gt;"",M26/$B$4*1000,IF(L26&lt;&gt;"",($A26-L26)/$B$4*1000,""))</f>
         <v/>
@@ -2592,8 +2592,8 @@
       <c r="P26" s="9" t="n">
         <v>1.9888</v>
       </c>
-      <c r="Q26" s="7" t="n"/>
-      <c r="R26" s="7" t="n"/>
+      <c r="Q26" s="7" t="inlineStr"/>
+      <c r="R26" s="7" t="inlineStr"/>
       <c r="S26" s="8">
         <f>IF(R26&lt;&gt;"",R26/$B$4*1000,IF(Q26&lt;&gt;"",($A26-Q26)/$B$4*1000,""))</f>
         <v/>
@@ -2609,8 +2609,8 @@
       <c r="A27" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="7" t="n"/>
+      <c r="B27" s="7" t="inlineStr"/>
+      <c r="C27" s="7" t="inlineStr"/>
       <c r="D27" s="8">
         <f>IF(C27&lt;&gt;"",C27/$B$4*1000,IF(B27&lt;&gt;"",($A27-B27)/$B$4*1000,""))</f>
         <v/>
@@ -2621,8 +2621,8 @@
       <c r="F27" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G27" s="7" t="n"/>
-      <c r="H27" s="7" t="n"/>
+      <c r="G27" s="7" t="inlineStr"/>
+      <c r="H27" s="7" t="inlineStr"/>
       <c r="I27" s="8">
         <f>IF(H27&lt;&gt;"",H27/$B$4*1000,IF(G27&lt;&gt;"",($A27-G27)/$B$4*1000,""))</f>
         <v/>
@@ -2633,8 +2633,8 @@
       <c r="K27" s="9" t="n">
         <v>0.4436</v>
       </c>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
+      <c r="L27" s="7" t="inlineStr"/>
+      <c r="M27" s="7" t="inlineStr"/>
       <c r="N27" s="8">
         <f>IF(M27&lt;&gt;"",M27/$B$4*1000,IF(L27&lt;&gt;"",($A27-L27)/$B$4*1000,""))</f>
         <v/>
@@ -2645,8 +2645,8 @@
       <c r="P27" s="9" t="n">
         <v>1.9981</v>
       </c>
-      <c r="Q27" s="7" t="n"/>
-      <c r="R27" s="7" t="n"/>
+      <c r="Q27" s="7" t="inlineStr"/>
+      <c r="R27" s="7" t="inlineStr"/>
       <c r="S27" s="8">
         <f>IF(R27&lt;&gt;"",R27/$B$4*1000,IF(Q27&lt;&gt;"",($A27-Q27)/$B$4*1000,""))</f>
         <v/>
@@ -2662,8 +2662,8 @@
       <c r="A28" s="6" t="n">
         <v>7.5</v>
       </c>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="n"/>
+      <c r="B28" s="7" t="inlineStr"/>
+      <c r="C28" s="7" t="inlineStr"/>
       <c r="D28" s="8">
         <f>IF(C28&lt;&gt;"",C28/$B$4*1000,IF(B28&lt;&gt;"",($A28-B28)/$B$4*1000,""))</f>
         <v/>
@@ -2674,8 +2674,8 @@
       <c r="F28" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G28" s="7" t="n"/>
-      <c r="H28" s="7" t="n"/>
+      <c r="G28" s="7" t="inlineStr"/>
+      <c r="H28" s="7" t="inlineStr"/>
       <c r="I28" s="8">
         <f>IF(H28&lt;&gt;"",H28/$B$4*1000,IF(G28&lt;&gt;"",($A28-G28)/$B$4*1000,""))</f>
         <v/>
@@ -2686,8 +2686,8 @@
       <c r="K28" s="9" t="n">
         <v>0.4457</v>
       </c>
-      <c r="L28" s="7" t="n"/>
-      <c r="M28" s="7" t="n"/>
+      <c r="L28" s="7" t="inlineStr"/>
+      <c r="M28" s="7" t="inlineStr"/>
       <c r="N28" s="8">
         <f>IF(M28&lt;&gt;"",M28/$B$4*1000,IF(L28&lt;&gt;"",($A28-L28)/$B$4*1000,""))</f>
         <v/>
@@ -2698,8 +2698,8 @@
       <c r="P28" s="9" t="n">
         <v>2.0074</v>
       </c>
-      <c r="Q28" s="7" t="n"/>
-      <c r="R28" s="7" t="n"/>
+      <c r="Q28" s="7" t="inlineStr"/>
+      <c r="R28" s="7" t="inlineStr"/>
       <c r="S28" s="8">
         <f>IF(R28&lt;&gt;"",R28/$B$4*1000,IF(Q28&lt;&gt;"",($A28-Q28)/$B$4*1000,""))</f>
         <v/>
@@ -2715,8 +2715,8 @@
       <c r="A29" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="n"/>
+      <c r="B29" s="7" t="inlineStr"/>
+      <c r="C29" s="7" t="inlineStr"/>
       <c r="D29" s="8">
         <f>IF(C29&lt;&gt;"",C29/$B$4*1000,IF(B29&lt;&gt;"",($A29-B29)/$B$4*1000,""))</f>
         <v/>
@@ -2727,8 +2727,8 @@
       <c r="F29" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G29" s="7" t="n"/>
-      <c r="H29" s="7" t="n"/>
+      <c r="G29" s="7" t="inlineStr"/>
+      <c r="H29" s="7" t="inlineStr"/>
       <c r="I29" s="8">
         <f>IF(H29&lt;&gt;"",H29/$B$4*1000,IF(G29&lt;&gt;"",($A29-G29)/$B$4*1000,""))</f>
         <v/>
@@ -2739,8 +2739,8 @@
       <c r="K29" s="9" t="n">
         <v>0.4477</v>
       </c>
-      <c r="L29" s="7" t="n"/>
-      <c r="M29" s="7" t="n"/>
+      <c r="L29" s="7" t="inlineStr"/>
+      <c r="M29" s="7" t="inlineStr"/>
       <c r="N29" s="8">
         <f>IF(M29&lt;&gt;"",M29/$B$4*1000,IF(L29&lt;&gt;"",($A29-L29)/$B$4*1000,""))</f>
         <v/>
@@ -2751,8 +2751,8 @@
       <c r="P29" s="9" t="n">
         <v>2.0168</v>
       </c>
-      <c r="Q29" s="7" t="n"/>
-      <c r="R29" s="7" t="n"/>
+      <c r="Q29" s="7" t="inlineStr"/>
+      <c r="R29" s="7" t="inlineStr"/>
       <c r="S29" s="8">
         <f>IF(R29&lt;&gt;"",R29/$B$4*1000,IF(Q29&lt;&gt;"",($A29-Q29)/$B$4*1000,""))</f>
         <v/>
@@ -2768,8 +2768,8 @@
       <c r="A30" s="6" t="n">
         <v>8.5</v>
       </c>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="7" t="n"/>
+      <c r="B30" s="7" t="inlineStr"/>
+      <c r="C30" s="7" t="inlineStr"/>
       <c r="D30" s="8">
         <f>IF(C30&lt;&gt;"",C30/$B$4*1000,IF(B30&lt;&gt;"",($A30-B30)/$B$4*1000,""))</f>
         <v/>
@@ -2780,8 +2780,8 @@
       <c r="F30" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="n"/>
+      <c r="G30" s="7" t="inlineStr"/>
+      <c r="H30" s="7" t="inlineStr"/>
       <c r="I30" s="8">
         <f>IF(H30&lt;&gt;"",H30/$B$4*1000,IF(G30&lt;&gt;"",($A30-G30)/$B$4*1000,""))</f>
         <v/>
@@ -2792,8 +2792,8 @@
       <c r="K30" s="9" t="n">
         <v>0.4498</v>
       </c>
-      <c r="L30" s="7" t="n"/>
-      <c r="M30" s="7" t="n"/>
+      <c r="L30" s="7" t="inlineStr"/>
+      <c r="M30" s="7" t="inlineStr"/>
       <c r="N30" s="8">
         <f>IF(M30&lt;&gt;"",M30/$B$4*1000,IF(L30&lt;&gt;"",($A30-L30)/$B$4*1000,""))</f>
         <v/>
@@ -2804,8 +2804,8 @@
       <c r="P30" s="9" t="n">
         <v>2.0261</v>
       </c>
-      <c r="Q30" s="7" t="n"/>
-      <c r="R30" s="7" t="n"/>
+      <c r="Q30" s="7" t="inlineStr"/>
+      <c r="R30" s="7" t="inlineStr"/>
       <c r="S30" s="8">
         <f>IF(R30&lt;&gt;"",R30/$B$4*1000,IF(Q30&lt;&gt;"",($A30-Q30)/$B$4*1000,""))</f>
         <v/>
@@ -2821,8 +2821,8 @@
       <c r="A31" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="7" t="n"/>
+      <c r="B31" s="7" t="inlineStr"/>
+      <c r="C31" s="7" t="inlineStr"/>
       <c r="D31" s="8">
         <f>IF(C31&lt;&gt;"",C31/$B$4*1000,IF(B31&lt;&gt;"",($A31-B31)/$B$4*1000,""))</f>
         <v/>
@@ -2833,8 +2833,8 @@
       <c r="F31" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
+      <c r="G31" s="7" t="inlineStr"/>
+      <c r="H31" s="7" t="inlineStr"/>
       <c r="I31" s="8">
         <f>IF(H31&lt;&gt;"",H31/$B$4*1000,IF(G31&lt;&gt;"",($A31-G31)/$B$4*1000,""))</f>
         <v/>
@@ -2845,8 +2845,8 @@
       <c r="K31" s="9" t="n">
         <v>0.4519</v>
       </c>
-      <c r="L31" s="7" t="n"/>
-      <c r="M31" s="7" t="n"/>
+      <c r="L31" s="7" t="inlineStr"/>
+      <c r="M31" s="7" t="inlineStr"/>
       <c r="N31" s="8">
         <f>IF(M31&lt;&gt;"",M31/$B$4*1000,IF(L31&lt;&gt;"",($A31-L31)/$B$4*1000,""))</f>
         <v/>
@@ -2857,8 +2857,8 @@
       <c r="P31" s="9" t="n">
         <v>2.0354</v>
       </c>
-      <c r="Q31" s="7" t="n"/>
-      <c r="R31" s="7" t="n"/>
+      <c r="Q31" s="7" t="inlineStr"/>
+      <c r="R31" s="7" t="inlineStr"/>
       <c r="S31" s="8">
         <f>IF(R31&lt;&gt;"",R31/$B$4*1000,IF(Q31&lt;&gt;"",($A31-Q31)/$B$4*1000,""))</f>
         <v/>
@@ -2874,8 +2874,8 @@
       <c r="A32" s="6" t="n">
         <v>9.5</v>
       </c>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="n"/>
+      <c r="B32" s="7" t="inlineStr"/>
+      <c r="C32" s="7" t="inlineStr"/>
       <c r="D32" s="8">
         <f>IF(C32&lt;&gt;"",C32/$B$4*1000,IF(B32&lt;&gt;"",($A32-B32)/$B$4*1000,""))</f>
         <v/>
@@ -2886,8 +2886,8 @@
       <c r="F32" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G32" s="7" t="n"/>
-      <c r="H32" s="7" t="n"/>
+      <c r="G32" s="7" t="inlineStr"/>
+      <c r="H32" s="7" t="inlineStr"/>
       <c r="I32" s="8">
         <f>IF(H32&lt;&gt;"",H32/$B$4*1000,IF(G32&lt;&gt;"",($A32-G32)/$B$4*1000,""))</f>
         <v/>
@@ -2898,8 +2898,8 @@
       <c r="K32" s="9" t="n">
         <v>0.454</v>
       </c>
-      <c r="L32" s="7" t="n"/>
-      <c r="M32" s="7" t="n"/>
+      <c r="L32" s="7" t="inlineStr"/>
+      <c r="M32" s="7" t="inlineStr"/>
       <c r="N32" s="8">
         <f>IF(M32&lt;&gt;"",M32/$B$4*1000,IF(L32&lt;&gt;"",($A32-L32)/$B$4*1000,""))</f>
         <v/>
@@ -2910,8 +2910,8 @@
       <c r="P32" s="9" t="n">
         <v>2.0448</v>
       </c>
-      <c r="Q32" s="7" t="n"/>
-      <c r="R32" s="7" t="n"/>
+      <c r="Q32" s="7" t="inlineStr"/>
+      <c r="R32" s="7" t="inlineStr"/>
       <c r="S32" s="8">
         <f>IF(R32&lt;&gt;"",R32/$B$4*1000,IF(Q32&lt;&gt;"",($A32-Q32)/$B$4*1000,""))</f>
         <v/>
@@ -2927,8 +2927,8 @@
       <c r="A33" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="7" t="n"/>
+      <c r="B33" s="7" t="inlineStr"/>
+      <c r="C33" s="7" t="inlineStr"/>
       <c r="D33" s="8">
         <f>IF(C33&lt;&gt;"",C33/$B$4*1000,IF(B33&lt;&gt;"",($A33-B33)/$B$4*1000,""))</f>
         <v/>
@@ -2939,8 +2939,8 @@
       <c r="F33" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G33" s="7" t="n"/>
-      <c r="H33" s="7" t="n"/>
+      <c r="G33" s="7" t="inlineStr"/>
+      <c r="H33" s="7" t="inlineStr"/>
       <c r="I33" s="8">
         <f>IF(H33&lt;&gt;"",H33/$B$4*1000,IF(G33&lt;&gt;"",($A33-G33)/$B$4*1000,""))</f>
         <v/>
@@ -2951,8 +2951,8 @@
       <c r="K33" s="9" t="n">
         <v>0.4561</v>
       </c>
-      <c r="L33" s="7" t="n"/>
-      <c r="M33" s="7" t="n"/>
+      <c r="L33" s="7" t="inlineStr"/>
+      <c r="M33" s="7" t="inlineStr"/>
       <c r="N33" s="8">
         <f>IF(M33&lt;&gt;"",M33/$B$4*1000,IF(L33&lt;&gt;"",($A33-L33)/$B$4*1000,""))</f>
         <v/>
@@ -2963,8 +2963,8 @@
       <c r="P33" s="9" t="n">
         <v>2.0541</v>
       </c>
-      <c r="Q33" s="7" t="n"/>
-      <c r="R33" s="7" t="n"/>
+      <c r="Q33" s="7" t="inlineStr"/>
+      <c r="R33" s="7" t="inlineStr"/>
       <c r="S33" s="8">
         <f>IF(R33&lt;&gt;"",R33/$B$4*1000,IF(Q33&lt;&gt;"",($A33-Q33)/$B$4*1000,""))</f>
         <v/>
@@ -2980,8 +2980,8 @@
       <c r="A34" s="6" t="n">
         <v>10.5</v>
       </c>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n"/>
+      <c r="B34" s="7" t="inlineStr"/>
+      <c r="C34" s="7" t="inlineStr"/>
       <c r="D34" s="8">
         <f>IF(C34&lt;&gt;"",C34/$B$4*1000,IF(B34&lt;&gt;"",($A34-B34)/$B$4*1000,""))</f>
         <v/>
@@ -2992,8 +2992,8 @@
       <c r="F34" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G34" s="7" t="n"/>
-      <c r="H34" s="7" t="n"/>
+      <c r="G34" s="7" t="inlineStr"/>
+      <c r="H34" s="7" t="inlineStr"/>
       <c r="I34" s="8">
         <f>IF(H34&lt;&gt;"",H34/$B$4*1000,IF(G34&lt;&gt;"",($A34-G34)/$B$4*1000,""))</f>
         <v/>
@@ -3004,8 +3004,8 @@
       <c r="K34" s="9" t="n">
         <v>0.4581</v>
       </c>
-      <c r="L34" s="7" t="n"/>
-      <c r="M34" s="7" t="n"/>
+      <c r="L34" s="7" t="inlineStr"/>
+      <c r="M34" s="7" t="inlineStr"/>
       <c r="N34" s="8">
         <f>IF(M34&lt;&gt;"",M34/$B$4*1000,IF(L34&lt;&gt;"",($A34-L34)/$B$4*1000,""))</f>
         <v/>
@@ -3016,8 +3016,8 @@
       <c r="P34" s="9" t="n">
         <v>2.0634</v>
       </c>
-      <c r="Q34" s="7" t="n"/>
-      <c r="R34" s="7" t="n"/>
+      <c r="Q34" s="7" t="inlineStr"/>
+      <c r="R34" s="7" t="inlineStr"/>
       <c r="S34" s="8">
         <f>IF(R34&lt;&gt;"",R34/$B$4*1000,IF(Q34&lt;&gt;"",($A34-Q34)/$B$4*1000,""))</f>
         <v/>
@@ -3033,8 +3033,8 @@
       <c r="A35" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="n"/>
+      <c r="B35" s="7" t="inlineStr"/>
+      <c r="C35" s="7" t="inlineStr"/>
       <c r="D35" s="8">
         <f>IF(C35&lt;&gt;"",C35/$B$4*1000,IF(B35&lt;&gt;"",($A35-B35)/$B$4*1000,""))</f>
         <v/>
@@ -3045,8 +3045,8 @@
       <c r="F35" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="G35" s="7" t="n"/>
-      <c r="H35" s="7" t="n"/>
+      <c r="G35" s="7" t="inlineStr"/>
+      <c r="H35" s="7" t="inlineStr"/>
       <c r="I35" s="8">
         <f>IF(H35&lt;&gt;"",H35/$B$4*1000,IF(G35&lt;&gt;"",($A35-G35)/$B$4*1000,""))</f>
         <v/>
@@ -3057,8 +3057,8 @@
       <c r="K35" s="9" t="n">
         <v>0.4602</v>
       </c>
-      <c r="L35" s="7" t="n"/>
-      <c r="M35" s="7" t="n"/>
+      <c r="L35" s="7" t="inlineStr"/>
+      <c r="M35" s="7" t="inlineStr"/>
       <c r="N35" s="8">
         <f>IF(M35&lt;&gt;"",M35/$B$4*1000,IF(L35&lt;&gt;"",($A35-L35)/$B$4*1000,""))</f>
         <v/>
@@ -3069,8 +3069,8 @@
       <c r="P35" s="9" t="n">
         <v>2.0727</v>
       </c>
-      <c r="Q35" s="7" t="n"/>
-      <c r="R35" s="7" t="n"/>
+      <c r="Q35" s="7" t="inlineStr"/>
+      <c r="R35" s="7" t="inlineStr"/>
       <c r="S35" s="8">
         <f>IF(R35&lt;&gt;"",R35/$B$4*1000,IF(Q35&lt;&gt;"",($A35-Q35)/$B$4*1000,""))</f>
         <v/>
@@ -3086,8 +3086,8 @@
       <c r="A36" s="6" t="n">
         <v>11.5</v>
       </c>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
+      <c r="B36" s="7" t="inlineStr"/>
+      <c r="C36" s="7" t="inlineStr"/>
       <c r="D36" s="8">
         <f>IF(C36&lt;&gt;"",C36/$B$4*1000,IF(B36&lt;&gt;"",($A36-B36)/$B$4*1000,""))</f>
         <v/>
@@ -3098,8 +3098,8 @@
       <c r="F36" s="9" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G36" s="7" t="n"/>
-      <c r="H36" s="7" t="n"/>
+      <c r="G36" s="7" t="inlineStr"/>
+      <c r="H36" s="7" t="inlineStr"/>
       <c r="I36" s="8">
         <f>IF(H36&lt;&gt;"",H36/$B$4*1000,IF(G36&lt;&gt;"",($A36-G36)/$B$4*1000,""))</f>
         <v/>
@@ -3110,8 +3110,8 @@
       <c r="K36" s="9" t="n">
         <v>0.4623</v>
       </c>
-      <c r="L36" s="7" t="n"/>
-      <c r="M36" s="7" t="n"/>
+      <c r="L36" s="7" t="inlineStr"/>
+      <c r="M36" s="7" t="inlineStr"/>
       <c r="N36" s="8">
         <f>IF(M36&lt;&gt;"",M36/$B$4*1000,IF(L36&lt;&gt;"",($A36-L36)/$B$4*1000,""))</f>
         <v/>
@@ -3122,8 +3122,8 @@
       <c r="P36" s="9" t="n">
         <v>2.0821</v>
       </c>
-      <c r="Q36" s="7" t="n"/>
-      <c r="R36" s="7" t="n"/>
+      <c r="Q36" s="7" t="inlineStr"/>
+      <c r="R36" s="7" t="inlineStr"/>
       <c r="S36" s="8">
         <f>IF(R36&lt;&gt;"",R36/$B$4*1000,IF(Q36&lt;&gt;"",($A36-Q36)/$B$4*1000,""))</f>
         <v/>
@@ -3139,8 +3139,8 @@
       <c r="A37" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="7" t="n"/>
+      <c r="B37" s="7" t="inlineStr"/>
+      <c r="C37" s="7" t="inlineStr"/>
       <c r="D37" s="8">
         <f>IF(C37&lt;&gt;"",C37/$B$4*1000,IF(B37&lt;&gt;"",($A37-B37)/$B$4*1000,""))</f>
         <v/>
@@ -3151,8 +3151,8 @@
       <c r="F37" s="9" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G37" s="7" t="n"/>
-      <c r="H37" s="7" t="n"/>
+      <c r="G37" s="7" t="inlineStr"/>
+      <c r="H37" s="7" t="inlineStr"/>
       <c r="I37" s="8">
         <f>IF(H37&lt;&gt;"",H37/$B$4*1000,IF(G37&lt;&gt;"",($A37-G37)/$B$4*1000,""))</f>
         <v/>
@@ -3163,8 +3163,8 @@
       <c r="K37" s="9" t="n">
         <v>0.4644</v>
       </c>
-      <c r="L37" s="7" t="n"/>
-      <c r="M37" s="7" t="n"/>
+      <c r="L37" s="7" t="inlineStr"/>
+      <c r="M37" s="7" t="inlineStr"/>
       <c r="N37" s="8">
         <f>IF(M37&lt;&gt;"",M37/$B$4*1000,IF(L37&lt;&gt;"",($A37-L37)/$B$4*1000,""))</f>
         <v/>
@@ -3175,8 +3175,8 @@
       <c r="P37" s="9" t="n">
         <v>2.0914</v>
       </c>
-      <c r="Q37" s="7" t="n"/>
-      <c r="R37" s="7" t="n"/>
+      <c r="Q37" s="7" t="inlineStr"/>
+      <c r="R37" s="7" t="inlineStr"/>
       <c r="S37" s="8">
         <f>IF(R37&lt;&gt;"",R37/$B$4*1000,IF(Q37&lt;&gt;"",($A37-Q37)/$B$4*1000,""))</f>
         <v/>
@@ -3192,8 +3192,8 @@
       <c r="A38" s="6" t="n">
         <v>12.5</v>
       </c>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="n"/>
+      <c r="B38" s="7" t="inlineStr"/>
+      <c r="C38" s="7" t="inlineStr"/>
       <c r="D38" s="8">
         <f>IF(C38&lt;&gt;"",C38/$B$4*1000,IF(B38&lt;&gt;"",($A38-B38)/$B$4*1000,""))</f>
         <v/>
@@ -3204,8 +3204,8 @@
       <c r="F38" s="9" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G38" s="7" t="n"/>
-      <c r="H38" s="7" t="n"/>
+      <c r="G38" s="7" t="inlineStr"/>
+      <c r="H38" s="7" t="inlineStr"/>
       <c r="I38" s="8">
         <f>IF(H38&lt;&gt;"",H38/$B$4*1000,IF(G38&lt;&gt;"",($A38-G38)/$B$4*1000,""))</f>
         <v/>
@@ -3216,8 +3216,8 @@
       <c r="K38" s="9" t="n">
         <v>0.4665</v>
       </c>
-      <c r="L38" s="7" t="n"/>
-      <c r="M38" s="7" t="n"/>
+      <c r="L38" s="7" t="inlineStr"/>
+      <c r="M38" s="7" t="inlineStr"/>
       <c r="N38" s="8">
         <f>IF(M38&lt;&gt;"",M38/$B$4*1000,IF(L38&lt;&gt;"",($A38-L38)/$B$4*1000,""))</f>
         <v/>
@@ -3228,8 +3228,8 @@
       <c r="P38" s="9" t="n">
         <v>2.1007</v>
       </c>
-      <c r="Q38" s="7" t="n"/>
-      <c r="R38" s="7" t="n"/>
+      <c r="Q38" s="7" t="inlineStr"/>
+      <c r="R38" s="7" t="inlineStr"/>
       <c r="S38" s="8">
         <f>IF(R38&lt;&gt;"",R38/$B$4*1000,IF(Q38&lt;&gt;"",($A38-Q38)/$B$4*1000,""))</f>
         <v/>
@@ -3245,8 +3245,8 @@
       <c r="A39" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="7" t="n"/>
+      <c r="B39" s="7" t="inlineStr"/>
+      <c r="C39" s="7" t="inlineStr"/>
       <c r="D39" s="8">
         <f>IF(C39&lt;&gt;"",C39/$B$4*1000,IF(B39&lt;&gt;"",($A39-B39)/$B$4*1000,""))</f>
         <v/>
@@ -3257,8 +3257,8 @@
       <c r="F39" s="9" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G39" s="7" t="n"/>
-      <c r="H39" s="7" t="n"/>
+      <c r="G39" s="7" t="inlineStr"/>
+      <c r="H39" s="7" t="inlineStr"/>
       <c r="I39" s="8">
         <f>IF(H39&lt;&gt;"",H39/$B$4*1000,IF(G39&lt;&gt;"",($A39-G39)/$B$4*1000,""))</f>
         <v/>
@@ -3269,8 +3269,8 @@
       <c r="K39" s="9" t="n">
         <v>0.4685</v>
       </c>
-      <c r="L39" s="7" t="n"/>
-      <c r="M39" s="7" t="n"/>
+      <c r="L39" s="7" t="inlineStr"/>
+      <c r="M39" s="7" t="inlineStr"/>
       <c r="N39" s="8">
         <f>IF(M39&lt;&gt;"",M39/$B$4*1000,IF(L39&lt;&gt;"",($A39-L39)/$B$4*1000,""))</f>
         <v/>
@@ -3281,8 +3281,8 @@
       <c r="P39" s="9" t="n">
         <v>2.11</v>
       </c>
-      <c r="Q39" s="7" t="n"/>
-      <c r="R39" s="7" t="n"/>
+      <c r="Q39" s="7" t="inlineStr"/>
+      <c r="R39" s="7" t="inlineStr"/>
       <c r="S39" s="8">
         <f>IF(R39&lt;&gt;"",R39/$B$4*1000,IF(Q39&lt;&gt;"",($A39-Q39)/$B$4*1000,""))</f>
         <v/>
@@ -3298,8 +3298,8 @@
       <c r="A40" s="6" t="n">
         <v>13.5</v>
       </c>
-      <c r="B40" s="7" t="n"/>
-      <c r="C40" s="7" t="n"/>
+      <c r="B40" s="7" t="inlineStr"/>
+      <c r="C40" s="7" t="inlineStr"/>
       <c r="D40" s="8">
         <f>IF(C40&lt;&gt;"",C40/$B$4*1000,IF(B40&lt;&gt;"",($A40-B40)/$B$4*1000,""))</f>
         <v/>
@@ -3310,8 +3310,8 @@
       <c r="F40" s="9" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G40" s="7" t="n"/>
-      <c r="H40" s="7" t="n"/>
+      <c r="G40" s="7" t="inlineStr"/>
+      <c r="H40" s="7" t="inlineStr"/>
       <c r="I40" s="8">
         <f>IF(H40&lt;&gt;"",H40/$B$4*1000,IF(G40&lt;&gt;"",($A40-G40)/$B$4*1000,""))</f>
         <v/>
@@ -3322,8 +3322,8 @@
       <c r="K40" s="9" t="n">
         <v>0.4706</v>
       </c>
-      <c r="L40" s="7" t="n"/>
-      <c r="M40" s="7" t="n"/>
+      <c r="L40" s="7" t="inlineStr"/>
+      <c r="M40" s="7" t="inlineStr"/>
       <c r="N40" s="8">
         <f>IF(M40&lt;&gt;"",M40/$B$4*1000,IF(L40&lt;&gt;"",($A40-L40)/$B$4*1000,""))</f>
         <v/>
@@ -3334,8 +3334,8 @@
       <c r="P40" s="9" t="n">
         <v>2.1194</v>
       </c>
-      <c r="Q40" s="7" t="n"/>
-      <c r="R40" s="7" t="n"/>
+      <c r="Q40" s="7" t="inlineStr"/>
+      <c r="R40" s="7" t="inlineStr"/>
       <c r="S40" s="8">
         <f>IF(R40&lt;&gt;"",R40/$B$4*1000,IF(Q40&lt;&gt;"",($A40-Q40)/$B$4*1000,""))</f>
         <v/>
@@ -3351,8 +3351,8 @@
       <c r="A41" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B41" s="7" t="n"/>
-      <c r="C41" s="7" t="n"/>
+      <c r="B41" s="7" t="inlineStr"/>
+      <c r="C41" s="7" t="inlineStr"/>
       <c r="D41" s="8">
         <f>IF(C41&lt;&gt;"",C41/$B$4*1000,IF(B41&lt;&gt;"",($A41-B41)/$B$4*1000,""))</f>
         <v/>
@@ -3363,8 +3363,8 @@
       <c r="F41" s="9" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G41" s="7" t="n"/>
-      <c r="H41" s="7" t="n"/>
+      <c r="G41" s="7" t="inlineStr"/>
+      <c r="H41" s="7" t="inlineStr"/>
       <c r="I41" s="8">
         <f>IF(H41&lt;&gt;"",H41/$B$4*1000,IF(G41&lt;&gt;"",($A41-G41)/$B$4*1000,""))</f>
         <v/>
@@ -3375,8 +3375,8 @@
       <c r="K41" s="9" t="n">
         <v>0.4727</v>
       </c>
-      <c r="L41" s="7" t="n"/>
-      <c r="M41" s="7" t="n"/>
+      <c r="L41" s="7" t="inlineStr"/>
+      <c r="M41" s="7" t="inlineStr"/>
       <c r="N41" s="8">
         <f>IF(M41&lt;&gt;"",M41/$B$4*1000,IF(L41&lt;&gt;"",($A41-L41)/$B$4*1000,""))</f>
         <v/>
@@ -3387,8 +3387,8 @@
       <c r="P41" s="9" t="n">
         <v>2.1287</v>
       </c>
-      <c r="Q41" s="7" t="n"/>
-      <c r="R41" s="7" t="n"/>
+      <c r="Q41" s="7" t="inlineStr"/>
+      <c r="R41" s="7" t="inlineStr"/>
       <c r="S41" s="8">
         <f>IF(R41&lt;&gt;"",R41/$B$4*1000,IF(Q41&lt;&gt;"",($A41-Q41)/$B$4*1000,""))</f>
         <v/>
@@ -3404,8 +3404,8 @@
       <c r="A42" s="6" t="n">
         <v>14.5</v>
       </c>
-      <c r="B42" s="7" t="n"/>
-      <c r="C42" s="7" t="n"/>
+      <c r="B42" s="7" t="inlineStr"/>
+      <c r="C42" s="7" t="inlineStr"/>
       <c r="D42" s="8">
         <f>IF(C42&lt;&gt;"",C42/$B$4*1000,IF(B42&lt;&gt;"",($A42-B42)/$B$4*1000,""))</f>
         <v/>
@@ -3416,8 +3416,8 @@
       <c r="F42" s="9" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G42" s="7" t="n"/>
-      <c r="H42" s="7" t="n"/>
+      <c r="G42" s="7" t="inlineStr"/>
+      <c r="H42" s="7" t="inlineStr"/>
       <c r="I42" s="8">
         <f>IF(H42&lt;&gt;"",H42/$B$4*1000,IF(G42&lt;&gt;"",($A42-G42)/$B$4*1000,""))</f>
         <v/>
@@ -3428,8 +3428,8 @@
       <c r="K42" s="9" t="n">
         <v>0.4748</v>
       </c>
-      <c r="L42" s="7" t="n"/>
-      <c r="M42" s="7" t="n"/>
+      <c r="L42" s="7" t="inlineStr"/>
+      <c r="M42" s="7" t="inlineStr"/>
       <c r="N42" s="8">
         <f>IF(M42&lt;&gt;"",M42/$B$4*1000,IF(L42&lt;&gt;"",($A42-L42)/$B$4*1000,""))</f>
         <v/>
@@ -3440,8 +3440,8 @@
       <c r="P42" s="9" t="n">
         <v>2.138</v>
       </c>
-      <c r="Q42" s="7" t="n"/>
-      <c r="R42" s="7" t="n"/>
+      <c r="Q42" s="7" t="inlineStr"/>
+      <c r="R42" s="7" t="inlineStr"/>
       <c r="S42" s="8">
         <f>IF(R42&lt;&gt;"",R42/$B$4*1000,IF(Q42&lt;&gt;"",($A42-Q42)/$B$4*1000,""))</f>
         <v/>
@@ -3457,8 +3457,8 @@
       <c r="A43" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B43" s="7" t="n"/>
-      <c r="C43" s="7" t="n"/>
+      <c r="B43" s="7" t="inlineStr"/>
+      <c r="C43" s="7" t="inlineStr"/>
       <c r="D43" s="8">
         <f>IF(C43&lt;&gt;"",C43/$B$4*1000,IF(B43&lt;&gt;"",($A43-B43)/$B$4*1000,""))</f>
         <v/>
@@ -3469,8 +3469,8 @@
       <c r="F43" s="9" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G43" s="7" t="n"/>
-      <c r="H43" s="7" t="n"/>
+      <c r="G43" s="7" t="inlineStr"/>
+      <c r="H43" s="7" t="inlineStr"/>
       <c r="I43" s="8">
         <f>IF(H43&lt;&gt;"",H43/$B$4*1000,IF(G43&lt;&gt;"",($A43-G43)/$B$4*1000,""))</f>
         <v/>
@@ -3481,8 +3481,8 @@
       <c r="K43" s="9" t="n">
         <v>0.4768</v>
       </c>
-      <c r="L43" s="7" t="n"/>
-      <c r="M43" s="7" t="n"/>
+      <c r="L43" s="7" t="inlineStr"/>
+      <c r="M43" s="7" t="inlineStr"/>
       <c r="N43" s="8">
         <f>IF(M43&lt;&gt;"",M43/$B$4*1000,IF(L43&lt;&gt;"",($A43-L43)/$B$4*1000,""))</f>
         <v/>
@@ -3493,8 +3493,8 @@
       <c r="P43" s="9" t="n">
         <v>2.1473</v>
       </c>
-      <c r="Q43" s="7" t="n"/>
-      <c r="R43" s="7" t="n"/>
+      <c r="Q43" s="7" t="inlineStr"/>
+      <c r="R43" s="7" t="inlineStr"/>
       <c r="S43" s="8">
         <f>IF(R43&lt;&gt;"",R43/$B$4*1000,IF(Q43&lt;&gt;"",($A43-Q43)/$B$4*1000,""))</f>
         <v/>
@@ -3550,7 +3550,7 @@
           <t>麵包板全景照 1 張</t>
         </is>
       </c>
-      <c r="B50" s="18" t="n"/>
+      <c r="B50" s="18" t="inlineStr"/>
       <c r="C50" s="19" t="inlineStr">
         <is>
           <t>看得出 R1／R2／RC 各插在第幾欄、電晶體三腳的 E／B／C 方向</t>
@@ -3563,7 +3563,7 @@
           <t>電表接線特寫 1 張</t>
         </is>
       </c>
-      <c r="B51" s="18" t="n"/>
+      <c r="B51" s="18" t="inlineStr"/>
       <c r="C51" s="19" t="inlineStr">
         <is>
           <t>左表跨 B-E、中表跨 C-E、右表設 DC 電壓檔並跨 RC 兩端量 V_RC</t>
@@ -3576,7 +3576,7 @@
           <t>兩台電源面板各 1 張</t>
         </is>
       </c>
-      <c r="B52" s="18" t="n"/>
+      <c r="B52" s="18" t="inlineStr"/>
       <c r="C52" s="19" t="inlineStr">
         <is>
           <t>V_BB 與 V_CC 的設定值要和記錄表對得上</t>
@@ -3589,7 +3589,7 @@
           <t>四組 V_BB 的 V_BE 都記到</t>
         </is>
       </c>
-      <c r="B53" s="18" t="n"/>
+      <c r="B53" s="18" t="inlineStr"/>
       <c r="C53" s="19" t="inlineStr">
         <is>
           <t>導通後 V_BE 幾乎不動，沒記到就無法回答「ON/OFF 怎麼判定」</t>
@@ -3602,7 +3602,7 @@
           <t>特性曲線當場畫一次</t>
         </is>
       </c>
-      <c r="B54" s="18" t="n"/>
+      <c r="B54" s="18" t="inlineStr"/>
       <c r="C54" s="19" t="inlineStr">
         <is>
           <t>四條線要看得出平坦的主動區；不平坦代表還沒離開飽和區</t>
@@ -4094,7 +4094,7 @@
           <t>R1 兩端壓降 V_R1</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
+      <c r="B7" s="7" t="inlineStr"/>
       <c r="C7" s="17" t="inlineStr">
         <is>
           <t>V</t>
@@ -4120,7 +4120,7 @@
           <t>R2 兩端壓降 V_R2</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
+      <c r="B8" s="7" t="inlineStr"/>
       <c r="C8" s="17" t="inlineStr">
         <is>
           <t>V</t>
@@ -4146,7 +4146,7 @@
           <t>R_C 兩端壓降 V_RC</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
+      <c r="B9" s="7" t="inlineStr"/>
       <c r="C9" s="17" t="inlineStr">
         <is>
           <t>V</t>
@@ -4172,7 +4172,7 @@
           <t>V_CE</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
+      <c r="B10" s="7" t="inlineStr"/>
       <c r="C10" s="17" t="inlineStr">
         <is>
           <t>V</t>
@@ -4363,7 +4363,7 @@
           <t>β_measure（三用電表 hFE 檔）</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
+      <c r="B16" s="7" t="inlineStr"/>
       <c r="C16" s="17" t="inlineStr">
         <is>
           <t>—</t>
@@ -4418,7 +4418,7 @@
           <t>四個壓降都量到</t>
         </is>
       </c>
-      <c r="B22" s="18" t="n"/>
+      <c r="B22" s="18" t="inlineStr"/>
       <c r="C22" s="19" t="inlineStr">
         <is>
           <t>V_R1、V_R2、V_RC、V_CE（V_CE 要直接量，不要相減）</t>
@@ -4431,7 +4431,7 @@
           <t>五個設定值都記下</t>
         </is>
       </c>
-      <c r="B23" s="18" t="n"/>
+      <c r="B23" s="18" t="inlineStr"/>
       <c r="C23" s="19" t="inlineStr">
         <is>
           <t>V_BB、V_CC 與 R1／R2／R_C 的實測值，助教要求</t>
@@ -4444,7 +4444,7 @@
           <t>Table 2 三欄填完</t>
         </is>
       </c>
-      <c r="B24" s="18" t="n"/>
+      <c r="B24" s="18" t="inlineStr"/>
       <c r="C24" s="19" t="inlineStr">
         <is>
           <t>講義 Table 2 只要 I_B、I_C、β_calculate（β_Meas 已被助教劃掉）</t>
@@ -4457,7 +4457,7 @@
           <t>電晶體 hFE 讀值照片 1 張</t>
         </is>
       </c>
-      <c r="B25" s="18" t="n"/>
+      <c r="B25" s="18" t="inlineStr"/>
       <c r="C25" s="19" t="inlineStr">
         <is>
           <t>拔下來插 hFE 座量到的 β，寫自己的記錄表、不抄進 Table 2</t>
@@ -4470,7 +4470,7 @@
           <t>飽和的證據 1 張</t>
         </is>
       </c>
-      <c r="B26" s="18" t="n"/>
+      <c r="B26" s="18" t="inlineStr"/>
       <c r="C26" s="19" t="inlineStr">
         <is>
           <t>V_CE 只剩幾十 mV 的電表畫面</t>
@@ -4606,7 +4606,7 @@
           <t>V_B（基極對地）</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
+      <c r="B6" s="7" t="inlineStr"/>
       <c r="C6" s="9" t="n">
         <v>5.876</v>
       </c>
@@ -4614,7 +4614,7 @@
         <f>IF(OR(B6="",C6=0),"",(B6-C6)/C6)</f>
         <v/>
       </c>
-      <c r="E6" s="7" t="n"/>
+      <c r="E6" s="7" t="inlineStr"/>
       <c r="F6" s="9" t="n">
         <v>5.87</v>
       </c>
@@ -4634,7 +4634,7 @@
           <t>V_E（射極對地）</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
+      <c r="B7" s="7" t="inlineStr"/>
       <c r="C7" s="9" t="n">
         <v>5.178</v>
       </c>
@@ -4642,7 +4642,7 @@
         <f>IF(OR(B7="",C7=0),"",(B7-C7)/C7)</f>
         <v/>
       </c>
-      <c r="E7" s="7" t="n"/>
+      <c r="E7" s="7" t="inlineStr"/>
       <c r="F7" s="9" t="n">
         <v>5.171</v>
       </c>
@@ -4662,7 +4662,7 @@
           <t>V_C（集極對地）</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
+      <c r="B8" s="7" t="inlineStr"/>
       <c r="C8" s="9" t="n">
         <v>11.485</v>
       </c>
@@ -4670,7 +4670,7 @@
         <f>IF(OR(B8="",C8=0),"",(B8-C8)/C8)</f>
         <v/>
       </c>
-      <c r="E8" s="7" t="n"/>
+      <c r="E8" s="7" t="inlineStr"/>
       <c r="F8" s="9" t="n">
         <v>6.854</v>
       </c>
@@ -4802,8 +4802,8 @@
           <t>RC1 100 Ω、有 C3</t>
         </is>
       </c>
-      <c r="B14" s="24" t="n"/>
-      <c r="C14" s="24" t="n"/>
+      <c r="B14" s="24" t="inlineStr"/>
+      <c r="C14" s="24" t="inlineStr"/>
       <c r="D14" s="25">
         <f>IF(OR(B14="",B14=0,C14=""),"",C14/B14)</f>
         <v/>
@@ -4815,7 +4815,7 @@
         <f>IF(OR(D14="",E14=0),"",(D14-E14)/E14)</f>
         <v/>
       </c>
-      <c r="G14" s="18" t="n"/>
+      <c r="G14" s="18" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
@@ -4823,8 +4823,8 @@
           <t>RC1 1 kΩ、有 C3</t>
         </is>
       </c>
-      <c r="B15" s="24" t="n"/>
-      <c r="C15" s="24" t="n"/>
+      <c r="B15" s="24" t="inlineStr"/>
+      <c r="C15" s="24" t="inlineStr"/>
       <c r="D15" s="25">
         <f>IF(OR(B15="",B15=0,C15=""),"",C15/B15)</f>
         <v/>
@@ -4836,7 +4836,7 @@
         <f>IF(OR(D15="",E15=0),"",(D15-E15)/E15)</f>
         <v/>
       </c>
-      <c r="G15" s="18" t="n"/>
+      <c r="G15" s="18" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
@@ -4844,8 +4844,8 @@
           <t>RC1 100 Ω、無 C3</t>
         </is>
       </c>
-      <c r="B16" s="24" t="n"/>
-      <c r="C16" s="24" t="n"/>
+      <c r="B16" s="24" t="inlineStr"/>
+      <c r="C16" s="24" t="inlineStr"/>
       <c r="D16" s="25">
         <f>IF(OR(B16="",B16=0,C16=""),"",C16/B16)</f>
         <v/>
@@ -4857,7 +4857,7 @@
         <f>IF(OR(D16="",E16=0),"",(D16-E16)/E16)</f>
         <v/>
       </c>
-      <c r="G16" s="18" t="n"/>
+      <c r="G16" s="18" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -4865,8 +4865,8 @@
           <t>RC1 1 kΩ、無 C3</t>
         </is>
       </c>
-      <c r="B17" s="24" t="n"/>
-      <c r="C17" s="24" t="n"/>
+      <c r="B17" s="24" t="inlineStr"/>
+      <c r="C17" s="24" t="inlineStr"/>
       <c r="D17" s="25">
         <f>IF(OR(B17="",B17=0,C17=""),"",C17/B17)</f>
         <v/>
@@ -4878,7 +4878,7 @@
         <f>IF(OR(D17="",E17=0),"",(D17-E17)/E17)</f>
         <v/>
       </c>
-      <c r="G17" s="18" t="n"/>
+      <c r="G17" s="18" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4939,7 +4939,7 @@
           <t>增益正比於集極端總電阻；620 Ω 剛好把 |A_v| 拉到 20</t>
         </is>
       </c>
-      <c r="D22" s="18" t="n"/>
+      <c r="D22" s="18" t="inlineStr"/>
       <c r="E22" s="12" t="n"/>
     </row>
     <row r="23">
@@ -4958,7 +4958,7 @@
           <t>留一小段不被旁路，增益改由電阻比決定，對 β 與溫度不敏感</t>
         </is>
       </c>
-      <c r="D23" s="18" t="n"/>
+      <c r="D23" s="18" t="inlineStr"/>
       <c r="E23" s="12" t="n"/>
     </row>
     <row r="24">
@@ -4977,7 +4977,7 @@
           <t>直流偏壓照舊由它決定，工作點不動</t>
         </is>
       </c>
-      <c r="D24" s="18" t="n"/>
+      <c r="D24" s="18" t="inlineStr"/>
       <c r="E24" s="12" t="n"/>
     </row>
     <row r="25">
@@ -4996,7 +4996,7 @@
           <t>10 kHz 時容抗 0.16 Ω，遠小於 R_E1a，才算真的旁路掉</t>
         </is>
       </c>
-      <c r="D25" s="18" t="n"/>
+      <c r="D25" s="18" t="inlineStr"/>
       <c r="E25" s="12" t="n"/>
     </row>
     <row r="26">
@@ -5015,7 +5015,7 @@
           <t>耦合電容維持講義原值即可，截止頻率遠低於 10 kHz</t>
         </is>
       </c>
-      <c r="D26" s="18" t="n"/>
+      <c r="D26" s="18" t="inlineStr"/>
       <c r="E26" s="12" t="n"/>
     </row>
     <row r="27">
@@ -5034,7 +5034,7 @@
           <t>工作點</t>
         </is>
       </c>
-      <c r="D27" s="18" t="n"/>
+      <c r="D27" s="18" t="inlineStr"/>
       <c r="E27" s="12" t="inlineStr">
         <is>
           <t>5.88 / 5.18 / 8.87 V</t>
@@ -5057,7 +5057,7 @@
           <t>目標 20，±10% 以內都算達標</t>
         </is>
       </c>
-      <c r="D28" s="18" t="n"/>
+      <c r="D28" s="18" t="inlineStr"/>
       <c r="E28" s="12" t="n">
         <v>20.13</v>
       </c>
@@ -5099,7 +5099,7 @@
           <t>示波器雙軌畫面 4 張</t>
         </is>
       </c>
-      <c r="B33" s="18" t="n"/>
+      <c r="B33" s="18" t="inlineStr"/>
       <c r="C33" s="19" t="inlineStr">
         <is>
           <t>四種組合各一張，CH1／CH2 同時入鏡才看得出反相</t>
@@ -5112,7 +5112,7 @@
           <t>削波的那張要放大</t>
         </is>
       </c>
-      <c r="B34" s="18" t="n"/>
+      <c r="B34" s="18" t="inlineStr"/>
       <c r="C34" s="19" t="inlineStr">
         <is>
           <t>R_C1 = 1 kΩ 的輸出，削平的一邊要看得清楚</t>
@@ -5125,7 +5125,7 @@
           <t>直流工作點電表照片 1 張</t>
         </is>
       </c>
-      <c r="B35" s="18" t="n"/>
+      <c r="B35" s="18" t="inlineStr"/>
       <c r="C35" s="19" t="inlineStr">
         <is>
           <t>V_B、V_E、V_C 三個讀值</t>
@@ -5138,7 +5138,7 @@
           <t>Bonus 電路的接線照與波形各 1 張</t>
         </is>
       </c>
-      <c r="B36" s="18" t="n"/>
+      <c r="B36" s="18" t="inlineStr"/>
       <c r="C36" s="19" t="inlineStr">
         <is>
           <t>元件值改了要拍，結報要對照</t>

</xml_diff>